<commit_message>
Added bulk delete + xlsx support for imports of journeys changed planninground steps
</commit_message>
<xml_diff>
--- a/reizen_2027.xlsx
+++ b/reizen_2027.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Reizen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,20 +16,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD-MM-YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,10 +48,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -421,66 +416,48 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Naam</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Startdatum</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Einddatum</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Bussen</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Reizigers</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Status (0=Huidig)</t>
-        </is>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Spanje Voorjaar</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n">
+        <v>46453</v>
+      </c>
+      <c r="C1" s="1" t="n">
+        <v>46463</v>
+      </c>
+      <c r="D1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E1" t="n">
+        <v>12</v>
+      </c>
+      <c r="F1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Spanje Voorjaar</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>46453</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>46463</v>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>46467</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>46477</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -489,20 +466,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>46467</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>46477</v>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>46481</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>46491</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -511,20 +488,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Marokko</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>46481</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>46491</v>
+          <t>Italië Voorjaar</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>46495</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>46505</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -533,20 +510,20 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Italië Voorjaar</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>46495</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>46505</v>
+          <t>Griekenland Lente</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>46509</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>46519</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -555,20 +532,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Griekenland Lente</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>46509</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>46519</v>
+          <t>Kroatië Lente</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>46523</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>46533</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -577,14 +554,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kroatië Lente</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>46523</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>46533</v>
+          <t>Turkije</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>46544</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>46554</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -599,20 +576,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Turkije</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>46544</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>46554</v>
+          <t>Spanje Zomer</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>46558</v>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>46568</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -621,14 +598,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Spanje Zomer</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>46558</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>46568</v>
+          <t>Italië Zomer</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>46572</v>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>46585</v>
       </c>
       <c r="D9" t="n">
         <v>2</v>
@@ -643,20 +620,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Italië Zomer</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>46572</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>46585</v>
+          <t>Griekenland Zomer</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>46587</v>
+      </c>
+      <c r="C10" s="1" t="n">
+        <v>46597</v>
       </c>
       <c r="D10" t="n">
         <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -665,20 +642,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Griekenland Zomer</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>46587</v>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>46597</v>
+          <t>Kroatië Zomer</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>46601</v>
+      </c>
+      <c r="C11" s="1" t="n">
+        <v>46611</v>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -687,20 +664,20 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Kroatië Zomer</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>46601</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>46611</v>
+          <t>Montenegro</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>46615</v>
+      </c>
+      <c r="C12" s="1" t="n">
+        <v>46625</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -709,20 +686,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Montenegro</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>46615</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>46625</v>
+          <t>Zwitserland</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>46635</v>
+      </c>
+      <c r="C13" s="1" t="n">
+        <v>46645</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -731,20 +708,20 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Zwitserland</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>46635</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>46645</v>
+          <t>Albanië</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>46649</v>
+      </c>
+      <c r="C14" s="1" t="n">
+        <v>46659</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -753,20 +730,20 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Albanië</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>46649</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>46659</v>
+          <t>Noorwegen</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>46663</v>
+      </c>
+      <c r="C15" s="1" t="n">
+        <v>46673</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -775,20 +752,20 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Noorwegen</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>46663</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>46673</v>
+          <t>IJsland</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>46677</v>
+      </c>
+      <c r="C16" s="1" t="n">
+        <v>46687</v>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -797,20 +774,20 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IJsland</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>46677</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>46687</v>
+          <t>Schotland</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>46691</v>
+      </c>
+      <c r="C17" s="1" t="n">
+        <v>46701</v>
       </c>
       <c r="D17" t="n">
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -819,44 +796,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Schotland</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>46691</v>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>46701</v>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="n">
+        <v>46705</v>
+      </c>
+      <c r="C18" s="1" t="n">
+        <v>46715</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Finland</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>46705</v>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>46715</v>
-      </c>
-      <c r="D19" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" t="n">
-        <v>8</v>
-      </c>
-      <c r="F19" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>